<commit_message>
Update app icon and quiz materials
</commit_message>
<xml_diff>
--- a/material_boki3.xlsx
+++ b/material_boki3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mr_sh\Desktop\bokiapp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5056013E-3655-42BB-84D8-693FB125E962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E00585-CA7E-48B8-8F04-640A24158D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE4C0FF7-C6FC-428E-A421-B60F5DF5D3D8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DE4C0FF7-C6FC-428E-A421-B60F5DF5D3D8}"/>
   </bookViews>
   <sheets>
     <sheet name="分類問題" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="171">
   <si>
     <t>answer_value</t>
   </si>
@@ -168,13 +168,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>応接セット、机、椅子、パソコン、ＦＡＸ、プリンター、コピ－機等</t>
-    <rPh sb="30" eb="31">
-      <t>トウ</t>
-    </rPh>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>借入金</t>
     <phoneticPr fontId="2"/>
   </si>
@@ -1465,6 +1458,682 @@
     </rPh>
     <rPh sb="12" eb="14">
       <t>ゼイキン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>応接セット、机、椅子、パソコン、プリンター、コピ－機等</t>
+    <rPh sb="26" eb="27">
+      <t>トウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>受取手数料</t>
+    <rPh sb="2" eb="5">
+      <t>テスウリョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>本業外で、仲介、斡旋、代行などにより受取った手数料</t>
+    <rPh sb="18" eb="20">
+      <t>ウケト</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>販売目的で商品を購入した際に使用する勘定科目</t>
+    <rPh sb="0" eb="2">
+      <t>ハンバイ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>モクテキ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ショウヒン</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>コウニュウ</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>サイ</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>シヨウ</t>
+    </rPh>
+    <rPh sb="18" eb="22">
+      <t>カンジョウカモク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売上原価</t>
+    <rPh sb="0" eb="4">
+      <t>ウリアゲゲンカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売れた（顧客に引渡した）商品の原価</t>
+    <rPh sb="0" eb="1">
+      <t>ウ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>コキャク</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ヒキワタ</t>
+    </rPh>
+    <rPh sb="12" eb="14">
+      <t>ショウヒン</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>ゲンカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>支払手数料</t>
+    <rPh sb="0" eb="2">
+      <t>シハライ</t>
+    </rPh>
+    <rPh sb="2" eb="5">
+      <t>テスウリョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>銀行振込、クレジットカード決済などのサービス利用時に外部に支払う際に使用する勘定科目</t>
+    <rPh sb="26" eb="28">
+      <t>ガイブ</t>
+    </rPh>
+    <rPh sb="29" eb="31">
+      <t>シハラ</t>
+    </rPh>
+    <rPh sb="32" eb="33">
+      <t>サイ</t>
+    </rPh>
+    <rPh sb="34" eb="36">
+      <t>シヨウ</t>
+    </rPh>
+    <rPh sb="38" eb="42">
+      <t>カンジョウカモク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>雑費</t>
+    <rPh sb="0" eb="2">
+      <t>ザッピ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>他のどの勘定科目にも当てはまらない、少額かつ一時的な出費</t>
+  </si>
+  <si>
+    <t>売掛金</t>
+    <rPh sb="0" eb="3">
+      <t>ウリカケキン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売上代金の未回収分で、後日受け取る予定のもの</t>
+    <rPh sb="0" eb="4">
+      <t>ウリアゲダイキン</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>ミカイシュウ</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>ブン</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ゴジツ</t>
+    </rPh>
+    <rPh sb="13" eb="14">
+      <t>ウ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>ト</t>
+    </rPh>
+    <rPh sb="17" eb="19">
+      <t>ヨテイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>仕入代金の未払い分で、後日支払う予定のもの</t>
+    <rPh sb="0" eb="2">
+      <t>シイ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ダイキン</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ミバラ</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>ブン</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ゴジツ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>シハラ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>ヨテイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>繰越商品</t>
+    <rPh sb="0" eb="4">
+      <t>クリコシショウヒン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>期末時点で販売されずに在庫として残っいる商品の原価</t>
+    <rPh sb="0" eb="4">
+      <t>キマツジテン</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ハンバイ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ザイコ</t>
+    </rPh>
+    <rPh sb="16" eb="17">
+      <t>ノコ</t>
+    </rPh>
+    <rPh sb="20" eb="22">
+      <t>ショウヒン</t>
+    </rPh>
+    <rPh sb="23" eb="25">
+      <t>ゲンカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>なぜ仕入は費用なのか？</t>
+    <rPh sb="2" eb="4">
+      <t>シイレ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ヒヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>テキストにそう書いてあるから</t>
+    <rPh sb="7" eb="8">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売上を得るために出て行ったことにするから</t>
+    <rPh sb="0" eb="2">
+      <t>ウリアゲ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>エ</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>デ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>イ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>なぜ繰越商品は資産なのか？</t>
+    <rPh sb="2" eb="6">
+      <t>クリコシショウヒン</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>シサン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>商品だから</t>
+    <rPh sb="0" eb="2">
+      <t>ショウヒン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>商品を仕入れたから</t>
+    <rPh sb="0" eb="2">
+      <t>ショウヒン</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>シイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>３分法を採用しているから</t>
+    <rPh sb="1" eb="2">
+      <t>ブン</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ホウ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>サイヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>３分法の場合、一旦すべて売れたことにして、期末に在庫を繰越商品として資産として処理します。</t>
+    <rPh sb="1" eb="3">
+      <t>ブンホウ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>バアイ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>イッタン</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>ウ</t>
+    </rPh>
+    <rPh sb="21" eb="23">
+      <t>キマツ</t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t>ザイコ</t>
+    </rPh>
+    <rPh sb="27" eb="31">
+      <t>クリコシショウヒン</t>
+    </rPh>
+    <rPh sb="34" eb="36">
+      <t>シサン</t>
+    </rPh>
+    <rPh sb="39" eb="41">
+      <t>ショリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売上原価対立法を採用しているから</t>
+    <rPh sb="0" eb="4">
+      <t>ウリアゲゲンカ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>タイリツ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>ホウ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>サイヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>お店の商品だから</t>
+    <rPh sb="1" eb="2">
+      <t>ミセ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ショウヒン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>期末時点で所有している在庫を表します。会社に残っているモノなので資産に該当します。</t>
+    <rPh sb="0" eb="2">
+      <t>キマツ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ジテン</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ショユウ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ザイコ</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>アラワ</t>
+    </rPh>
+    <rPh sb="19" eb="21">
+      <t>カイシャ</t>
+    </rPh>
+    <rPh sb="22" eb="23">
+      <t>ノコ</t>
+    </rPh>
+    <rPh sb="32" eb="34">
+      <t>シサン</t>
+    </rPh>
+    <rPh sb="35" eb="37">
+      <t>ガイトウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>まだその会社の商品だから</t>
+    <rPh sb="4" eb="6">
+      <t>カイシャ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ショウヒン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売れた商品の原価だから</t>
+    <rPh sb="0" eb="1">
+      <t>ウ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ショウヒン</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ゲンカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>まだ売上げていないから</t>
+    <rPh sb="2" eb="4">
+      <t>ウリア</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>なぜ消耗品を買うと費用なのか？</t>
+    <rPh sb="2" eb="5">
+      <t>ショウモウヒン</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>カ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ヒヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>まだ使っていないから</t>
+    <rPh sb="2" eb="3">
+      <t>ツカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>金額が少額で、資産計上する必要がないから</t>
+    <rPh sb="0" eb="2">
+      <t>キンガク</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ショウガク</t>
+    </rPh>
+    <rPh sb="7" eb="11">
+      <t>シサンケイジョウ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ヒツヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>これから使う文房具類だから</t>
+    <rPh sb="4" eb="5">
+      <t>ツカ</t>
+    </rPh>
+    <rPh sb="6" eb="9">
+      <t>ブンボウグ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>ルイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>使い切ったから</t>
+    <rPh sb="0" eb="1">
+      <t>ツカ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>キ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>消耗品も厳密には購入時は、会社の所有物ですが、使い切ることが明白で少額なので、消耗品費として費用処理します。</t>
+    <rPh sb="0" eb="3">
+      <t>ショウモウヒン</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ゲンミツ</t>
+    </rPh>
+    <rPh sb="8" eb="11">
+      <t>コウニュウジ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>カイシャ</t>
+    </rPh>
+    <rPh sb="16" eb="19">
+      <t>ショユウブツ</t>
+    </rPh>
+    <rPh sb="23" eb="24">
+      <t>ツカ</t>
+    </rPh>
+    <rPh sb="25" eb="26">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="30" eb="32">
+      <t>メイハク</t>
+    </rPh>
+    <rPh sb="33" eb="35">
+      <t>ショウガク</t>
+    </rPh>
+    <rPh sb="39" eb="43">
+      <t>ショウモウヒンヒ</t>
+    </rPh>
+    <rPh sb="46" eb="48">
+      <t>ヒヨウ</t>
+    </rPh>
+    <rPh sb="48" eb="50">
+      <t>ショリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>なぜ売掛金は資産なのか？</t>
+    <rPh sb="2" eb="5">
+      <t>ウリカケキン</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>シサン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売上代金で回収した分だから</t>
+    <rPh sb="0" eb="2">
+      <t>ウリアゲ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ダイキン</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>カイシュウ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>ブン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>将来、お客さんに請求できるから</t>
+    <rPh sb="0" eb="2">
+      <t>ショウライ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>キャク</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>セイキュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>将来、お客さんに請求されるから</t>
+    <rPh sb="0" eb="2">
+      <t>ショウライ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>キャク</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>セイキュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売掛金とは売上代金でまだお客さんからお金を頂いていない分で、将来請求し、お金に変わります。</t>
+    <rPh sb="0" eb="3">
+      <t>ウリカケキン</t>
+    </rPh>
+    <rPh sb="5" eb="9">
+      <t>ウリアゲダイキン</t>
+    </rPh>
+    <rPh sb="13" eb="14">
+      <t>キャク</t>
+    </rPh>
+    <rPh sb="19" eb="20">
+      <t>カネ</t>
+    </rPh>
+    <rPh sb="21" eb="22">
+      <t>イタダ</t>
+    </rPh>
+    <rPh sb="27" eb="28">
+      <t>ブン</t>
+    </rPh>
+    <rPh sb="30" eb="32">
+      <t>ショウライ</t>
+    </rPh>
+    <rPh sb="32" eb="34">
+      <t>セイキュウ</t>
+    </rPh>
+    <rPh sb="37" eb="38">
+      <t>カネ</t>
+    </rPh>
+    <rPh sb="39" eb="40">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>なぜ買掛金は負債なのか？</t>
+    <rPh sb="2" eb="5">
+      <t>カイカケキン</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>フサイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>売上代金だから</t>
+    <rPh sb="0" eb="2">
+      <t>ウリアゲ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ダイキン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>将来、支払う義務があるから</t>
+    <rPh sb="0" eb="2">
+      <t>ショウライ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>シハラ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ギム</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>将来、受取る権利があるから</t>
+    <rPh sb="0" eb="2">
+      <t>ショウライ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ウケト</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ケンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>将来の仕入だから</t>
+    <rPh sb="0" eb="2">
+      <t>ショウライ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>シイレ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>将来の売上だから</t>
+    <rPh sb="0" eb="2">
+      <t>ショウライ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ウリアゲ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>買掛金とは仕入代金でまだ仕入先に支払っていない分で、将来請求され、お金を支払います。</t>
+    <rPh sb="0" eb="3">
+      <t>カイカケキン</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>シイ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ダイキン</t>
+    </rPh>
+    <rPh sb="12" eb="14">
+      <t>シイレ</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>サキ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>シハラ</t>
+    </rPh>
+    <rPh sb="23" eb="24">
+      <t>ブン</t>
+    </rPh>
+    <rPh sb="26" eb="28">
+      <t>ショウライ</t>
+    </rPh>
+    <rPh sb="28" eb="30">
+      <t>セイキュウ</t>
+    </rPh>
+    <rPh sb="34" eb="35">
+      <t>カネ</t>
+    </rPh>
+    <rPh sb="36" eb="38">
+      <t>シハライ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -1473,7 +2142,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1535,6 +2204,21 @@
       <family val="1"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="ＭＳ 明朝"/>
+      <family val="1"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1558,7 +2242,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1588,6 +2272,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1923,7 +2613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0246E57E-1A7C-477B-962D-8E28C390228D}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="13.875" style="1" bestFit="1" customWidth="1"/>
@@ -1944,10 +2634,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
@@ -1958,10 +2648,10 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E2" s="1">
         <v>1</v>
@@ -1978,7 +2668,7 @@
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3" s="1">
         <v>2</v>
@@ -1995,7 +2685,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4" s="1">
         <v>1</v>
@@ -2012,7 +2702,7 @@
         <v>11</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" s="1">
         <v>1</v>
@@ -2029,7 +2719,7 @@
         <v>12</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" s="1">
         <v>1</v>
@@ -2040,13 +2730,13 @@
         <v>1</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="1">
         <v>1</v>
@@ -2060,10 +2750,10 @@
         <v>8</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>14</v>
+        <v>124</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8" s="1">
         <v>1</v>
@@ -2074,13 +2764,13 @@
         <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E9" s="1">
         <v>1</v>
@@ -2091,13 +2781,13 @@
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="D10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
@@ -2108,13 +2798,13 @@
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E11" s="1">
         <v>1</v>
@@ -2125,13 +2815,13 @@
         <v>4</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E12" s="1">
         <v>1</v>
@@ -2142,13 +2832,13 @@
         <v>4</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>25</v>
+        <v>19</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E13" s="1">
         <v>1</v>
@@ -2159,13 +2849,13 @@
         <v>5</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="D14" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E14" s="1">
         <v>1</v>
@@ -2176,13 +2866,13 @@
         <v>5</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>29</v>
-      </c>
       <c r="D15" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E15" s="1">
         <v>1</v>
@@ -2193,13 +2883,13 @@
         <v>5</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="D16" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E16" s="1">
         <v>1</v>
@@ -2210,10 +2900,11 @@
         <v>5</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>121</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="C17" s="10"/>
       <c r="D17" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E17" s="1">
         <v>3</v>
@@ -2224,10 +2915,11 @@
         <v>5</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>122</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="C18" s="10"/>
       <c r="D18" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E18" s="1">
         <v>3</v>
@@ -2238,17 +2930,555 @@
         <v>5</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="D19" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E19" s="1">
         <v>2</v>
       </c>
+    </row>
+    <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="1">
+        <v>4</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="1">
+        <v>5</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="1">
+        <v>5</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="1">
+        <v>5</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="1">
+        <v>5</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="1">
+        <v>1</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="1">
+        <v>2</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="1">
+        <v>1</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E27" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C28" s="10"/>
+    </row>
+    <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C29" s="10"/>
+    </row>
+    <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C30" s="10"/>
+    </row>
+    <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C31" s="10"/>
+    </row>
+    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C32" s="10"/>
+    </row>
+    <row r="33" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C33" s="10"/>
+    </row>
+    <row r="34" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C34" s="10"/>
+    </row>
+    <row r="35" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C35" s="10"/>
+    </row>
+    <row r="36" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C36" s="10"/>
+    </row>
+    <row r="37" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C37" s="10"/>
+    </row>
+    <row r="38" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C38" s="10"/>
+    </row>
+    <row r="39" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C39" s="10"/>
+    </row>
+    <row r="40" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C40" s="10"/>
+    </row>
+    <row r="41" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C41" s="10"/>
+    </row>
+    <row r="42" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C42" s="10"/>
+    </row>
+    <row r="43" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C43" s="10"/>
+    </row>
+    <row r="44" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C44" s="10"/>
+    </row>
+    <row r="45" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C45" s="10"/>
+    </row>
+    <row r="46" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C46" s="10"/>
+    </row>
+    <row r="47" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C47" s="10"/>
+    </row>
+    <row r="48" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C48" s="10"/>
+    </row>
+    <row r="49" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C49" s="10"/>
+    </row>
+    <row r="50" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C50" s="10"/>
+    </row>
+    <row r="51" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C51" s="10"/>
+    </row>
+    <row r="52" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C52" s="10"/>
+    </row>
+    <row r="53" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C53" s="10"/>
+    </row>
+    <row r="54" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C54" s="10"/>
+    </row>
+    <row r="55" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C55" s="10"/>
+    </row>
+    <row r="56" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C56" s="10"/>
+    </row>
+    <row r="57" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C57" s="10"/>
+    </row>
+    <row r="58" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C58" s="10"/>
+    </row>
+    <row r="59" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C59" s="10"/>
+    </row>
+    <row r="60" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C60" s="10"/>
+    </row>
+    <row r="61" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C61" s="10"/>
+    </row>
+    <row r="62" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C62" s="10"/>
+    </row>
+    <row r="63" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C63" s="10"/>
+    </row>
+    <row r="64" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C64" s="10"/>
+    </row>
+    <row r="65" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C65" s="10"/>
+    </row>
+    <row r="66" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C66" s="10"/>
+    </row>
+    <row r="67" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C67" s="10"/>
+    </row>
+    <row r="68" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C68" s="10"/>
+    </row>
+    <row r="69" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C69" s="10"/>
+    </row>
+    <row r="70" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C70" s="10"/>
+    </row>
+    <row r="71" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C71" s="10"/>
+    </row>
+    <row r="72" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C72" s="10"/>
+    </row>
+    <row r="73" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C73" s="10"/>
+    </row>
+    <row r="74" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C74" s="10"/>
+    </row>
+    <row r="75" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C75" s="10"/>
+    </row>
+    <row r="76" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C76" s="10"/>
+    </row>
+    <row r="77" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C77" s="10"/>
+    </row>
+    <row r="78" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C78" s="10"/>
+    </row>
+    <row r="79" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C79" s="10"/>
+    </row>
+    <row r="80" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C80" s="10"/>
+    </row>
+    <row r="81" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C81" s="10"/>
+    </row>
+    <row r="82" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C82" s="10"/>
+    </row>
+    <row r="83" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C83" s="10"/>
+    </row>
+    <row r="84" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C84" s="10"/>
+    </row>
+    <row r="85" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C85" s="10"/>
+    </row>
+    <row r="86" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C86" s="10"/>
+    </row>
+    <row r="87" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C87" s="10"/>
+    </row>
+    <row r="88" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C88" s="10"/>
+    </row>
+    <row r="89" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C89" s="10"/>
+    </row>
+    <row r="90" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C90" s="10"/>
+    </row>
+    <row r="91" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C91" s="10"/>
+    </row>
+    <row r="92" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C92" s="10"/>
+    </row>
+    <row r="93" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C93" s="10"/>
+    </row>
+    <row r="94" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C94" s="10"/>
+    </row>
+    <row r="95" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C95" s="10"/>
+    </row>
+    <row r="96" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C96" s="10"/>
+    </row>
+    <row r="97" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C97" s="10"/>
+    </row>
+    <row r="98" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C98" s="10"/>
+    </row>
+    <row r="99" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C99" s="10"/>
+    </row>
+    <row r="100" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C100" s="10"/>
+    </row>
+    <row r="101" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C101" s="10"/>
+    </row>
+    <row r="102" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C102" s="10"/>
+    </row>
+    <row r="103" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C103" s="10"/>
+    </row>
+    <row r="104" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C104" s="10"/>
+    </row>
+    <row r="105" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C105" s="10"/>
+    </row>
+    <row r="106" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C106" s="10"/>
+    </row>
+    <row r="107" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C107" s="10"/>
+    </row>
+    <row r="108" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C108" s="10"/>
+    </row>
+    <row r="109" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C109" s="10"/>
+    </row>
+    <row r="110" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C110" s="10"/>
+    </row>
+    <row r="111" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C111" s="10"/>
+    </row>
+    <row r="112" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C112" s="10"/>
+    </row>
+    <row r="113" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C113" s="10"/>
+    </row>
+    <row r="114" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C114" s="10"/>
+    </row>
+    <row r="115" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C115" s="10"/>
+    </row>
+    <row r="116" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C116" s="10"/>
+    </row>
+    <row r="117" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C117" s="10"/>
+    </row>
+    <row r="118" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C118" s="10"/>
+    </row>
+    <row r="119" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C119" s="10"/>
+    </row>
+    <row r="120" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C120" s="10"/>
+    </row>
+    <row r="121" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C121" s="10"/>
+    </row>
+    <row r="122" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C122" s="10"/>
+    </row>
+    <row r="123" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C123" s="10"/>
+    </row>
+    <row r="124" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C124" s="10"/>
+    </row>
+    <row r="125" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C125" s="10"/>
+    </row>
+    <row r="126" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C126" s="10"/>
+    </row>
+    <row r="127" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C127" s="10"/>
+    </row>
+    <row r="128" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C128" s="10"/>
+    </row>
+    <row r="129" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C129" s="10"/>
+    </row>
+    <row r="130" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C130" s="10"/>
+    </row>
+    <row r="131" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C131" s="10"/>
+    </row>
+    <row r="132" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C132" s="10"/>
+    </row>
+    <row r="133" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C133" s="10"/>
+    </row>
+    <row r="134" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C134" s="10"/>
+    </row>
+    <row r="135" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C135" s="10"/>
+    </row>
+    <row r="136" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C136" s="10"/>
+    </row>
+    <row r="137" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C137" s="10"/>
+    </row>
+    <row r="138" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C138" s="10"/>
+    </row>
+    <row r="139" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C139" s="10"/>
+    </row>
+    <row r="140" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C140" s="10"/>
+    </row>
+    <row r="141" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C141" s="10"/>
+    </row>
+    <row r="142" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C142" s="10"/>
+    </row>
+    <row r="143" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C143" s="10"/>
+    </row>
+    <row r="144" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C144" s="10"/>
+    </row>
+    <row r="145" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C145" s="10"/>
+    </row>
+    <row r="146" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C146" s="10"/>
+    </row>
+    <row r="147" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C147" s="10"/>
+    </row>
+    <row r="148" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C148" s="10"/>
+    </row>
+    <row r="149" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C149" s="10"/>
+    </row>
+    <row r="150" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C150" s="10"/>
+    </row>
+    <row r="151" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C151" s="10"/>
+    </row>
+    <row r="152" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C152" s="10"/>
+    </row>
+    <row r="153" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C153" s="10"/>
+    </row>
+    <row r="154" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C154" s="10"/>
+    </row>
+    <row r="155" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C155" s="10"/>
+    </row>
+    <row r="156" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C156" s="10"/>
+    </row>
+    <row r="157" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C157" s="10"/>
+    </row>
+    <row r="158" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C158" s="10"/>
+    </row>
+    <row r="159" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C159" s="10"/>
+    </row>
+    <row r="160" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C160" s="10"/>
+    </row>
+    <row r="161" spans="3:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C161" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -2258,61 +3488,64 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B52B2431-11E2-4394-A320-3C115695266D}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="27.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="117" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" t="s">
         <v>58</v>
-      </c>
-      <c r="B1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" t="s">
-        <v>59</v>
       </c>
       <c r="G1" t="s">
         <v>2</v>
       </c>
       <c r="H1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
         <v>42</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
         <v>43</v>
       </c>
-      <c r="C2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>44</v>
-      </c>
-      <c r="E2" t="s">
-        <v>45</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="G2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -2320,25 +3553,25 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" t="s">
         <v>48</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>49</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>50</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>51</v>
-      </c>
-      <c r="E3" t="s">
-        <v>52</v>
       </c>
       <c r="F3">
         <v>3</v>
       </c>
       <c r="G3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -2346,25 +3579,25 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" t="s">
         <v>54</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
         <v>55</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>51</v>
-      </c>
-      <c r="D4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" t="s">
-        <v>52</v>
       </c>
       <c r="F4">
         <v>2</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -2372,25 +3605,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s">
         <v>113</v>
       </c>
-      <c r="B5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>114</v>
-      </c>
-      <c r="E5" t="s">
-        <v>115</v>
       </c>
       <c r="F5">
         <v>3</v>
       </c>
       <c r="G5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H5">
         <v>3</v>
@@ -2398,28 +3631,184 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" t="s">
         <v>117</v>
       </c>
-      <c r="B6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" t="s">
-        <v>118</v>
-      </c>
       <c r="D6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E6" t="s">
         <v>114</v>
-      </c>
-      <c r="E6" t="s">
-        <v>115</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H6">
         <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" t="s">
+        <v>141</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
+        <v>146</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" t="s">
+        <v>151</v>
+      </c>
+      <c r="E8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>149</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C9" t="s">
+        <v>145</v>
+      </c>
+      <c r="D9" t="s">
+        <v>147</v>
+      </c>
+      <c r="E9" t="s">
+        <v>148</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9" t="s">
+        <v>146</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" t="s">
+        <v>156</v>
+      </c>
+      <c r="E10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" t="s">
+        <v>165</v>
+      </c>
+      <c r="C11" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" t="s">
+        <v>162</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11" t="s">
+        <v>163</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B12" t="s">
+        <v>166</v>
+      </c>
+      <c r="C12" t="s">
+        <v>167</v>
+      </c>
+      <c r="D12" t="s">
+        <v>168</v>
+      </c>
+      <c r="E12" t="s">
+        <v>169</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>170</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2438,54 +3827,54 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>59</v>
       </c>
-      <c r="G1" t="s">
-        <v>60</v>
-      </c>
       <c r="I1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A2" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" t="s">
         <v>61</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>62</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>63</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>64</v>
-      </c>
-      <c r="E2" t="s">
-        <v>65</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="G2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -2493,25 +3882,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
         <v>67</v>
-      </c>
-      <c r="B3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" t="s">
-        <v>68</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -2519,25 +3908,25 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A4" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" t="s">
         <v>69</v>
       </c>
-      <c r="B4" t="s">
-        <v>70</v>
-      </c>
       <c r="C4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" t="s">
         <v>86</v>
-      </c>
-      <c r="D4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E4" t="s">
-        <v>87</v>
       </c>
       <c r="F4">
         <v>3</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -2545,25 +3934,25 @@
     </row>
     <row r="5" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" t="s">
         <v>74</v>
-      </c>
-      <c r="D5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E5" t="s">
-        <v>75</v>
       </c>
       <c r="F5">
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -2571,25 +3960,25 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A6" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
         <v>79</v>
-      </c>
-      <c r="D6" t="s">
-        <v>82</v>
-      </c>
-      <c r="E6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
-        <v>80</v>
       </c>
       <c r="I6">
         <v>2</v>
@@ -2608,104 +3997,104 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" t="s">
         <v>90</v>
       </c>
-      <c r="C1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D1" t="s">
-        <v>89</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K1" t="s">
         <v>102</v>
       </c>
-      <c r="F1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1" t="s">
-        <v>92</v>
-      </c>
-      <c r="H1" t="s">
-        <v>93</v>
-      </c>
-      <c r="I1" t="s">
-        <v>94</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>95</v>
       </c>
-      <c r="K1" t="s">
-        <v>103</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>96</v>
       </c>
-      <c r="M1" t="s">
-        <v>97</v>
-      </c>
       <c r="N1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="O1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" t="s">
         <v>98</v>
-      </c>
-      <c r="B2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C2" t="s">
-        <v>99</v>
       </c>
       <c r="D2">
         <v>100000</v>
       </c>
       <c r="E2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G2">
         <v>30000</v>
       </c>
       <c r="K2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M2">
         <v>70000</v>
       </c>
       <c r="N2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" t="s">
         <v>109</v>
-      </c>
-      <c r="B3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C3" t="s">
-        <v>110</v>
       </c>
       <c r="D3">
         <v>100000</v>
       </c>
       <c r="E3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G3">
         <v>100000</v>
@@ -2713,22 +4102,22 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D4">
         <v>200000</v>
       </c>
       <c r="E4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G4">
         <v>200000</v>

</xml_diff>